<commit_message>
Gold v2: relabel under revised guide (rules R1-R4), log every change, keep v1
</commit_message>
<xml_diff>
--- a/labels/gold.xlsx
+++ b/labels/gold.xlsx
@@ -619,7 +619,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>more_info_requested</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>post_marketing</t>
+          <t>new_indication_or_change</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>post_marketing</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>clinical_trial</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>post_marketing</t>
+          <t>new_indication_or_change</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>more_info_requested</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>post_marketing</t>
+          <t>new_indication_or_change</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>approved_with_conditions</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>post_marketing</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>deferred</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>deferred</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -3204,7 +3204,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>deferred</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
@@ -3439,7 +3439,7 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>deferred</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
@@ -3523,7 +3523,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>bioequivalence</t>
+          <t>new_indication_or_change</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>more_info_requested</t>
+          <t>approved_with_conditions</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>deferred</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>post_marketing</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -3909,7 +3909,7 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>more_info_requested</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
@@ -4087,7 +4087,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>new_indication_or_change</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -4322,7 +4322,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>post_marketing</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -4473,7 +4473,7 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>approved_with_conditions</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>bioequivalence</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -4567,7 +4567,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>more_info_requested</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
@@ -4802,7 +4802,7 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>post_marketing</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -5262,7 +5262,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>clinical_trial</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -5272,7 +5272,7 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>post_marketing</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -5497,7 +5497,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>post_marketing</t>
+          <t>new_indication_or_change</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>approved_with_conditions</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr">
@@ -5685,7 +5685,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>post_marketing</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -5789,7 +5789,7 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr">
@@ -5967,7 +5967,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>post_marketing</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>bioequivalence</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -6447,7 +6447,7 @@
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="I128" s="2" t="inlineStr">
@@ -6541,7 +6541,7 @@
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="I130" s="2" t="inlineStr">
@@ -6729,7 +6729,7 @@
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="I134" s="2" t="inlineStr">
@@ -6766,7 +6766,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>clinical_trial</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -6776,7 +6776,7 @@
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="I135" s="2" t="inlineStr">
@@ -7001,7 +7001,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>clinical_trial</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -7011,7 +7011,7 @@
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>more_info_requested</t>
+          <t>approved_with_conditions</t>
         </is>
       </c>
       <c r="I140" s="2" t="inlineStr">
@@ -7105,7 +7105,7 @@
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="I142" s="2" t="inlineStr">
@@ -7199,7 +7199,7 @@
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>more_info_requested</t>
+          <t>approved_with_conditions</t>
         </is>
       </c>
       <c r="I144" s="2" t="inlineStr">
@@ -7236,7 +7236,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>clinical_trial</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -7246,7 +7246,7 @@
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="I145" s="2" t="inlineStr">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>clinical_trial</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -7293,7 +7293,7 @@
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="I146" s="2" t="inlineStr">
@@ -7387,7 +7387,7 @@
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>approved_with_conditions</t>
         </is>
       </c>
       <c r="I148" s="2" t="inlineStr">
@@ -7471,7 +7471,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>clinical_trial</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -7481,7 +7481,7 @@
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="I150" s="2" t="inlineStr">
@@ -7518,7 +7518,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>clinical_trial</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -7565,7 +7565,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>clinical_trial</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="I153" s="2" t="inlineStr">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>clinical_trial</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -7753,7 +7753,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>protocol_amendment</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -7763,7 +7763,7 @@
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="I156" s="2" t="inlineStr">
@@ -7800,7 +7800,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>clinical_trial</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -7847,7 +7847,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>protocol_amendment</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -7894,7 +7894,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>clinical_trial</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -8035,7 +8035,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>clinical_trial</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -8176,7 +8176,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>post_marketing</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -8270,7 +8270,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>post_marketing</t>
+          <t>new_indication_or_change</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -8327,7 +8327,7 @@
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="I168" s="2" t="inlineStr">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>clinical_trial</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -8421,7 +8421,7 @@
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>more_info_requested</t>
         </is>
       </c>
       <c r="I170" s="2" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>clinical_trial</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -8609,7 +8609,7 @@
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>more_info_requested</t>
         </is>
       </c>
       <c r="I174" s="2" t="inlineStr">
@@ -8750,7 +8750,7 @@
       </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>deferred</t>
         </is>
       </c>
       <c r="I177" s="2" t="inlineStr">
@@ -8928,7 +8928,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>clinical_trial</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -8938,7 +8938,7 @@
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="I181" s="2" t="inlineStr">
@@ -9116,7 +9116,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>clinical_trial</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -9210,7 +9210,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>clinical_trial</t>
+          <t>marketing_new_drug</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -9220,7 +9220,7 @@
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="I187" s="2" t="inlineStr">
@@ -9831,7 +9831,7 @@
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
-          <t>more_info_requested</t>
+          <t>rejected</t>
         </is>
       </c>
       <c r="I200" s="2" t="inlineStr">

</xml_diff>